<commit_message>
updated valus on 21st aug
</commit_message>
<xml_diff>
--- a/12600316.xlsx
+++ b/12600316.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piyus\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piyus\OneDrive\Desktop\cap776\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBC55827-20A2-4A6E-B829-8503277FB106}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{408925F2-1392-4633-9009-19CFDDE0CA44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="64">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -212,6 +212,21 @@
   </si>
   <si>
     <t>Optimist</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>motivated</t>
+  </si>
+  <si>
+    <t>Excellent</t>
+  </si>
+  <si>
+    <t>Very Satisfied</t>
+  </si>
+  <si>
+    <t>good</t>
   </si>
 </sst>
 </file>
@@ -1083,48 +1098,96 @@
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A8" s="13"/>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
-      <c r="I8" s="15" t="str">
+      <c r="A8" s="13">
+        <v>46254</v>
+      </c>
+      <c r="B8" s="14">
+        <v>480</v>
+      </c>
+      <c r="C8" s="14">
+        <v>30</v>
+      </c>
+      <c r="D8" s="14">
+        <v>130</v>
+      </c>
+      <c r="E8" s="14">
+        <v>300</v>
+      </c>
+      <c r="F8" s="14">
+        <v>200</v>
+      </c>
+      <c r="G8" s="14">
+        <v>4</v>
+      </c>
+      <c r="H8" s="14">
+        <v>300</v>
+      </c>
+      <c r="I8" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J8" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J8" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K8" s="16"/>
-      <c r="L8" s="16"/>
-      <c r="M8" s="16"/>
-      <c r="N8" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K8" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L8" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M8" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N8" s="17" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A9" s="13"/>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
-      <c r="H9" s="14"/>
-      <c r="I9" s="15" t="str">
+      <c r="A9" s="13">
+        <v>46255</v>
+      </c>
+      <c r="B9" s="14">
+        <v>400</v>
+      </c>
+      <c r="C9" s="14">
+        <v>30</v>
+      </c>
+      <c r="D9" s="14">
+        <v>350</v>
+      </c>
+      <c r="E9" s="14">
+        <v>300</v>
+      </c>
+      <c r="F9" s="14">
+        <v>200</v>
+      </c>
+      <c r="G9" s="14">
+        <v>4</v>
+      </c>
+      <c r="H9" s="14">
+        <v>160</v>
+      </c>
+      <c r="I9" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J9" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J9" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K9" s="16"/>
-      <c r="L9" s="16"/>
-      <c r="M9" s="16"/>
-      <c r="N9" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K9" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="L9" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="M9" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N9" s="17" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" s="13"/>

</xml_diff>

<commit_message>
update of 3rd Aug
</commit_message>
<xml_diff>
--- a/12600316.xlsx
+++ b/12600316.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piyus\OneDrive\Desktop\cap776\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67F57D5C-A45C-4E0F-9C42-6D99ECDDE726}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38397EF1-4FAF-4F85-A099-D635CDBAAC20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="77">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -205,9 +205,6 @@
     <t>Greatfull</t>
   </si>
   <si>
-    <t xml:space="preserve"> AUGUST</t>
-  </si>
-  <si>
     <t>High</t>
   </si>
   <si>
@@ -264,6 +261,12 @@
   <si>
     <t>improving myself day by day</t>
   </si>
+  <si>
+    <t>hostel room got boom</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> September</t>
+  </si>
 </sst>
 </file>
 
@@ -272,7 +275,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -353,6 +356,13 @@
       <name val="Arial"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -401,7 +411,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -445,6 +455,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -974,8 +985,8 @@
       <c r="E3" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="F3" s="20" t="s">
-        <v>56</v>
+      <c r="F3" s="21" t="s">
+        <v>76</v>
       </c>
       <c r="G3" s="20"/>
     </row>
@@ -1127,10 +1138,10 @@
         <v>50</v>
       </c>
       <c r="M7" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="N7" s="17" t="s">
         <v>57</v>
-      </c>
-      <c r="N7" s="17" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
@@ -1173,10 +1184,10 @@
         <v>50</v>
       </c>
       <c r="M8" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N8" s="17" t="s">
         <v>59</v>
-      </c>
-      <c r="N8" s="17" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
@@ -1213,16 +1224,16 @@
         <v>0</v>
       </c>
       <c r="K9" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="L9" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="L9" s="16" t="s">
+      <c r="M9" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="N9" s="17" t="s">
         <v>62</v>
-      </c>
-      <c r="M9" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="N9" s="17" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
@@ -1259,16 +1270,16 @@
         <v>560</v>
       </c>
       <c r="K10" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="L10" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="M10" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="N10" t="s">
         <v>64</v>
-      </c>
-      <c r="L10" s="16" t="s">
-        <v>64</v>
-      </c>
-      <c r="M10" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="N10" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
@@ -1305,16 +1316,16 @@
         <v>200</v>
       </c>
       <c r="K11" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="L11" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="L11" s="16" t="s">
-        <v>62</v>
-      </c>
       <c r="M11" s="16" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="N11" s="17" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
@@ -1351,16 +1362,16 @@
         <v>0</v>
       </c>
       <c r="K12" s="16" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="L12" s="16" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="M12" s="16" t="s">
         <v>54</v>
       </c>
       <c r="N12" s="17" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
@@ -1403,10 +1414,10 @@
         <v>50</v>
       </c>
       <c r="M13" s="16" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="N13" s="17" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
@@ -1449,10 +1460,10 @@
         <v>50</v>
       </c>
       <c r="M14" s="16" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="N14" s="17" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
@@ -1489,16 +1500,16 @@
         <v>0</v>
       </c>
       <c r="K15" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="L15" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="L15" s="16" t="s">
-        <v>62</v>
-      </c>
       <c r="M15" s="16" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="N15" s="17" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
@@ -1541,10 +1552,10 @@
         <v>50</v>
       </c>
       <c r="M16" s="16" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="N16" s="17" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">
@@ -1587,10 +1598,10 @@
         <v>50</v>
       </c>
       <c r="M17" s="16" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="N17" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
@@ -1630,13 +1641,13 @@
         <v>49</v>
       </c>
       <c r="L18" s="16" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="M18" s="16" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="N18" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.3">
@@ -1679,10 +1690,10 @@
         <v>50</v>
       </c>
       <c r="M19" s="16" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="N19" s="17" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
@@ -1719,61 +1730,109 @@
         <v>0</v>
       </c>
       <c r="K20" s="16" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="L20" s="16" t="s">
         <v>50</v>
       </c>
       <c r="M20" s="16" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="N20" s="17" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A21" s="13">
+        <v>46267</v>
+      </c>
+      <c r="B21" s="14">
+        <v>480</v>
+      </c>
+      <c r="C21" s="14">
+        <v>30</v>
+      </c>
+      <c r="D21" s="14">
+        <v>60</v>
+      </c>
+      <c r="E21" s="14">
+        <v>150</v>
+      </c>
+      <c r="F21" s="14">
+        <v>350</v>
+      </c>
+      <c r="G21" s="14">
+        <v>7</v>
+      </c>
+      <c r="H21" s="14">
+        <v>370</v>
+      </c>
+      <c r="I21" s="15">
+        <f>IF(SUM(B21:F21,H21)=0,"",SUM(B21:F21,H21))</f>
+        <v>1440</v>
+      </c>
+      <c r="J21" s="15">
+        <f>IF(I21="","",1440-I21)</f>
+        <v>0</v>
+      </c>
+      <c r="K21" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="L21" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="M21" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N21" s="17" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A21" s="13"/>
-      <c r="B21" s="14"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="14"/>
-      <c r="F21" s="14"/>
-      <c r="G21" s="14"/>
-      <c r="H21" s="14"/>
-      <c r="I21" s="15" t="str">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A22" s="13">
+        <v>46268</v>
+      </c>
+      <c r="B22" s="14">
+        <v>480</v>
+      </c>
+      <c r="C22" s="14">
+        <v>30</v>
+      </c>
+      <c r="D22" s="14">
+        <v>120</v>
+      </c>
+      <c r="E22" s="14">
+        <v>30</v>
+      </c>
+      <c r="F22" s="14">
+        <v>200</v>
+      </c>
+      <c r="G22" s="14">
+        <v>4</v>
+      </c>
+      <c r="H22" s="14">
+        <v>580</v>
+      </c>
+      <c r="I22" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J21" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J22" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K21" s="16"/>
-      <c r="L21" s="16"/>
-      <c r="M21" s="16"/>
-      <c r="N21" s="17"/>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A22" s="13"/>
-      <c r="B22" s="14"/>
-      <c r="C22" s="14"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="14"/>
-      <c r="F22" s="14"/>
-      <c r="G22" s="14"/>
-      <c r="H22" s="14"/>
-      <c r="I22" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J22" s="15" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K22" s="16"/>
-      <c r="L22" s="16"/>
-      <c r="M22" s="16"/>
-      <c r="N22" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K22" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="L22" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="M22" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N22" s="17" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" s="13"/>
@@ -10142,6 +10201,6 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update of 4th Aug
</commit_message>
<xml_diff>
--- a/12600316.xlsx
+++ b/12600316.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piyus\OneDrive\Desktop\cap776\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38397EF1-4FAF-4F85-A099-D635CDBAAC20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDB6D263-CF0A-4D27-868D-5DE92CB4CB6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="78">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -266,6 +266,9 @@
   </si>
   <si>
     <t xml:space="preserve"> September</t>
+  </si>
+  <si>
+    <t>R&amp;D for new project</t>
   </si>
 </sst>
 </file>
@@ -1835,26 +1838,50 @@
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A23" s="13"/>
-      <c r="B23" s="14"/>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="14"/>
-      <c r="F23" s="14"/>
-      <c r="G23" s="14"/>
-      <c r="H23" s="14"/>
-      <c r="I23" s="15" t="str">
+      <c r="A23" s="13">
+        <v>46269</v>
+      </c>
+      <c r="B23" s="14">
+        <v>480</v>
+      </c>
+      <c r="C23" s="14">
+        <v>30</v>
+      </c>
+      <c r="D23" s="14">
+        <v>120</v>
+      </c>
+      <c r="E23" s="14">
+        <v>180</v>
+      </c>
+      <c r="F23" s="14">
+        <v>250</v>
+      </c>
+      <c r="G23" s="14">
+        <v>5</v>
+      </c>
+      <c r="H23" s="14">
+        <v>380</v>
+      </c>
+      <c r="I23" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J23" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J23" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K23" s="16"/>
-      <c r="L23" s="16"/>
-      <c r="M23" s="16"/>
-      <c r="N23" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K23" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L23" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M23" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N23" s="17" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A24" s="13"/>

</xml_diff>

<commit_message>
update of 5th Aug
</commit_message>
<xml_diff>
--- a/12600316.xlsx
+++ b/12600316.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piyus\OneDrive\Desktop\cap776\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDB6D263-CF0A-4D27-868D-5DE92CB4CB6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3BD6A59-154E-4D87-8962-A5C19856771A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="79">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -269,6 +269,9 @@
   </si>
   <si>
     <t>R&amp;D for new project</t>
+  </si>
+  <si>
+    <t>new feature added to project</t>
   </si>
 </sst>
 </file>
@@ -1884,26 +1887,50 @@
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A24" s="13"/>
-      <c r="B24" s="14"/>
-      <c r="C24" s="14"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
-      <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
-      <c r="I24" s="15" t="str">
+      <c r="A24" s="13">
+        <v>46270</v>
+      </c>
+      <c r="B24" s="14">
+        <v>480</v>
+      </c>
+      <c r="C24" s="14">
+        <v>60</v>
+      </c>
+      <c r="D24" s="14">
+        <v>240</v>
+      </c>
+      <c r="E24" s="14">
+        <v>100</v>
+      </c>
+      <c r="F24" s="14">
+        <v>0</v>
+      </c>
+      <c r="G24" s="14">
+        <v>0</v>
+      </c>
+      <c r="H24" s="14">
+        <v>300</v>
+      </c>
+      <c r="I24" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J24" s="15" t="str">
+        <v>1180</v>
+      </c>
+      <c r="J24" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K24" s="16"/>
-      <c r="L24" s="16"/>
-      <c r="M24" s="16"/>
-      <c r="N24" s="17"/>
+        <v>260</v>
+      </c>
+      <c r="K24" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L24" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M24" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N24" s="17" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25" s="13"/>

</xml_diff>

<commit_message>
update of 7th & 8th Aug
</commit_message>
<xml_diff>
--- a/12600316.xlsx
+++ b/12600316.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piyus\OneDrive\Desktop\cap776\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{641F3089-928E-47E4-B8B8-03331C2658A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E33F2B96-7A40-4680-BD71-8F8189A5DCF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="82">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -275,6 +275,12 @@
   </si>
   <si>
     <t xml:space="preserve">improving </t>
+  </si>
+  <si>
+    <t>room shifting done</t>
+  </si>
+  <si>
+    <t>another productive day</t>
   </si>
 </sst>
 </file>
@@ -1982,48 +1988,96 @@
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A26" s="13"/>
-      <c r="B26" s="14"/>
-      <c r="C26" s="14"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14"/>
-      <c r="F26" s="14"/>
-      <c r="G26" s="14"/>
-      <c r="H26" s="14"/>
-      <c r="I26" s="15" t="str">
+      <c r="A26" s="13">
+        <v>46272</v>
+      </c>
+      <c r="B26" s="14">
+        <v>480</v>
+      </c>
+      <c r="C26" s="14">
+        <v>30</v>
+      </c>
+      <c r="D26" s="14">
+        <v>300</v>
+      </c>
+      <c r="E26" s="14">
+        <v>60</v>
+      </c>
+      <c r="F26" s="14">
+        <v>200</v>
+      </c>
+      <c r="G26" s="14">
+        <v>4</v>
+      </c>
+      <c r="H26" s="14">
+        <v>370</v>
+      </c>
+      <c r="I26" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J26" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J26" s="15">
+        <f>IF(I26="","",1440-I26)</f>
+        <v>0</v>
+      </c>
+      <c r="K26" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L26" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M26" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="N26" s="17" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A27" s="13">
+        <v>46273</v>
+      </c>
+      <c r="B27" s="14">
+        <v>480</v>
+      </c>
+      <c r="C27" s="14">
+        <v>30</v>
+      </c>
+      <c r="D27" s="14">
+        <v>180</v>
+      </c>
+      <c r="E27" s="14">
+        <v>200</v>
+      </c>
+      <c r="F27" s="14">
+        <v>350</v>
+      </c>
+      <c r="G27" s="14">
+        <v>7</v>
+      </c>
+      <c r="H27" s="14">
+        <v>200</v>
+      </c>
+      <c r="I27" s="15">
+        <f t="shared" si="0"/>
+        <v>1440</v>
+      </c>
+      <c r="J27" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K26" s="16"/>
-      <c r="L26" s="16"/>
-      <c r="M26" s="16"/>
-      <c r="N26" s="17"/>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A27" s="13"/>
-      <c r="B27" s="14"/>
-      <c r="C27" s="14"/>
-      <c r="D27" s="14"/>
-      <c r="E27" s="14"/>
-      <c r="F27" s="14"/>
-      <c r="G27" s="14"/>
-      <c r="H27" s="14"/>
-      <c r="I27" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J27" s="15" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K27" s="16"/>
-      <c r="L27" s="16"/>
-      <c r="M27" s="16"/>
-      <c r="N27" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K27" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="L27" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M27" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="N27" s="17" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A28" s="13"/>

</xml_diff>

<commit_message>
update of 10th Aug
</commit_message>
<xml_diff>
--- a/12600316.xlsx
+++ b/12600316.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piyus\OneDrive\Desktop\cap776\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E33F2B96-7A40-4680-BD71-8F8189A5DCF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8AAB789-01E0-46C9-A844-2D58A3C6B2D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="84">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -281,6 +281,12 @@
   </si>
   <si>
     <t>another productive day</t>
+  </si>
+  <si>
+    <t>lets do it</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fresher party </t>
   </si>
 </sst>
 </file>
@@ -2080,48 +2086,96 @@
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A28" s="13"/>
-      <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="14"/>
-      <c r="F28" s="14"/>
-      <c r="G28" s="14"/>
-      <c r="H28" s="14"/>
-      <c r="I28" s="15" t="str">
+      <c r="A28" s="13">
+        <v>46274</v>
+      </c>
+      <c r="B28" s="14">
+        <v>480</v>
+      </c>
+      <c r="C28" s="14">
+        <v>30</v>
+      </c>
+      <c r="D28" s="14">
+        <v>120</v>
+      </c>
+      <c r="E28" s="14">
+        <v>150</v>
+      </c>
+      <c r="F28" s="14">
+        <v>350</v>
+      </c>
+      <c r="G28" s="14">
+        <v>7</v>
+      </c>
+      <c r="H28" s="14">
+        <v>310</v>
+      </c>
+      <c r="I28" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J28" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J28" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K28" s="16"/>
-      <c r="L28" s="16"/>
-      <c r="M28" s="16"/>
-      <c r="N28" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K28" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L28" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M28" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N28" s="17" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A29" s="13"/>
-      <c r="B29" s="14"/>
-      <c r="C29" s="14"/>
-      <c r="D29" s="14"/>
-      <c r="E29" s="14"/>
-      <c r="F29" s="14"/>
-      <c r="G29" s="14"/>
-      <c r="H29" s="14"/>
-      <c r="I29" s="15" t="str">
+      <c r="A29" s="13">
+        <v>46275</v>
+      </c>
+      <c r="B29" s="14">
+        <v>480</v>
+      </c>
+      <c r="C29" s="14">
+        <v>30</v>
+      </c>
+      <c r="D29" s="14">
+        <v>240</v>
+      </c>
+      <c r="E29" s="14">
+        <v>60</v>
+      </c>
+      <c r="F29" s="14">
+        <v>200</v>
+      </c>
+      <c r="G29" s="14">
+        <v>4</v>
+      </c>
+      <c r="H29" s="14">
+        <v>200</v>
+      </c>
+      <c r="I29" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J29" s="15" t="str">
+        <v>1210</v>
+      </c>
+      <c r="J29" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K29" s="16"/>
-      <c r="L29" s="16"/>
-      <c r="M29" s="16"/>
-      <c r="N29" s="17"/>
+        <v>230</v>
+      </c>
+      <c r="K29" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L29" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M29" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N29" s="17" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A30" s="13"/>

</xml_diff>

<commit_message>
update of 12th Aug
</commit_message>
<xml_diff>
--- a/12600316.xlsx
+++ b/12600316.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piyus\OneDrive\Desktop\cap776\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8AAB789-01E0-46C9-A844-2D58A3C6B2D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F173810-A75F-420A-9609-C7EA78174514}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="86">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -287,6 +287,12 @@
   </si>
   <si>
     <t xml:space="preserve">fresher party </t>
+  </si>
+  <si>
+    <t>cyber security club discussion</t>
+  </si>
+  <si>
+    <t>team meeting done</t>
   </si>
 </sst>
 </file>
@@ -2178,48 +2184,96 @@
       </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A30" s="13"/>
-      <c r="B30" s="14"/>
-      <c r="C30" s="14"/>
-      <c r="D30" s="14"/>
-      <c r="E30" s="14"/>
-      <c r="F30" s="14"/>
-      <c r="G30" s="14"/>
-      <c r="H30" s="14"/>
-      <c r="I30" s="15" t="str">
+      <c r="A30" s="13">
+        <v>46276</v>
+      </c>
+      <c r="B30" s="14">
+        <v>480</v>
+      </c>
+      <c r="C30" s="14">
+        <v>30</v>
+      </c>
+      <c r="D30" s="14">
+        <v>180</v>
+      </c>
+      <c r="E30" s="14">
+        <v>100</v>
+      </c>
+      <c r="F30" s="14">
+        <v>250</v>
+      </c>
+      <c r="G30" s="14">
+        <v>5</v>
+      </c>
+      <c r="H30" s="14">
+        <v>400</v>
+      </c>
+      <c r="I30" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J30" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J30" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K30" s="16"/>
-      <c r="L30" s="16"/>
-      <c r="M30" s="16"/>
-      <c r="N30" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K30" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L30" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M30" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N30" s="17" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A31" s="13"/>
-      <c r="B31" s="14"/>
-      <c r="C31" s="14"/>
-      <c r="D31" s="14"/>
-      <c r="E31" s="14"/>
-      <c r="F31" s="14"/>
-      <c r="G31" s="14"/>
-      <c r="H31" s="14"/>
-      <c r="I31" s="15" t="str">
+      <c r="A31" s="13">
+        <v>46277</v>
+      </c>
+      <c r="B31" s="14">
+        <v>480</v>
+      </c>
+      <c r="C31" s="14">
+        <v>60</v>
+      </c>
+      <c r="D31" s="14">
+        <v>180</v>
+      </c>
+      <c r="E31" s="14">
+        <v>100</v>
+      </c>
+      <c r="F31" s="14">
+        <v>0</v>
+      </c>
+      <c r="G31" s="14">
+        <v>0</v>
+      </c>
+      <c r="H31" s="14">
+        <v>400</v>
+      </c>
+      <c r="I31" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J31" s="15" t="str">
+        <v>1220</v>
+      </c>
+      <c r="J31" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K31" s="16"/>
-      <c r="L31" s="16"/>
-      <c r="M31" s="16"/>
-      <c r="N31" s="17"/>
+        <v>220</v>
+      </c>
+      <c r="K31" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="L31" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="M31" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N31" s="17" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A32" s="13"/>

</xml_diff>